<commit_message>
Subo archivo modelos empezado
</commit_message>
<xml_diff>
--- a/hiperparam.xlsx
+++ b/hiperparam.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F5E12DE-E8E1-484A-8297-7F9815C1B417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163BF012-7FE1-414B-A428-538614F6DEF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34260" yWindow="1575" windowWidth="21600" windowHeight="11295" xr2:uid="{48A2C70B-EA9F-4526-AA9C-C7801D1D079C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{48A2C70B-EA9F-4526-AA9C-C7801D1D079C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>TABLA DE EXPERIMENTACIÓN DE HIPERPARÁMETROS</t>
   </si>
@@ -81,13 +81,31 @@
   </si>
   <si>
     <t>V1</t>
+  </si>
+  <si>
+    <t>V2</t>
+  </si>
+  <si>
+    <t>32, 16</t>
+  </si>
+  <si>
+    <t>16, 8</t>
+  </si>
+  <si>
+    <t>V3</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>(Conv1D) 32</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,8 +127,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -135,8 +161,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -204,7 +236,95 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
         <color indexed="64"/>
       </left>
       <right/>
@@ -213,14 +333,95 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thick">
         <color indexed="64"/>
       </left>
       <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top style="thick">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -229,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -242,8 +443,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -251,19 +450,40 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -665,7 +885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D926FC-4454-481D-AEC4-611B9C1DE27D}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
@@ -675,13 +895,13 @@
     <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -693,50 +913,50 @@
       <c r="G3" s="3"/>
       <c r="H3" s="4"/>
     </row>
-    <row r="4" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="K4" s="12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="25" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="5">
         <v>15</v>
       </c>
       <c r="C5" s="5">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D5" s="5">
         <v>32</v>
@@ -750,34 +970,165 @@
       <c r="G5" s="5">
         <v>1E-3</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="26">
         <v>18.25</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="15">
         <v>1.2522</v>
       </c>
-      <c r="J5" s="12">
+      <c r="J5" s="13">
         <v>0.98919999999999997</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="16">
         <v>0.95909999999999995</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="6"/>
+      <c r="B6" s="6">
+        <v>24</v>
+      </c>
+      <c r="C6" s="6">
+        <v>50</v>
+      </c>
+      <c r="D6" s="6">
+        <v>32</v>
+      </c>
+      <c r="E6" s="6">
+        <v>16</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="H6" s="21">
+        <v>18.25</v>
+      </c>
+      <c r="I6" s="17">
+        <v>1.3815999999999999</v>
+      </c>
+      <c r="J6" s="14">
+        <v>1.08683</v>
+      </c>
+      <c r="K6" s="18">
+        <v>0.95079999999999998</v>
+      </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="6">
+        <v>15</v>
+      </c>
+      <c r="C7" s="6">
+        <v>50</v>
+      </c>
+      <c r="D7" s="6">
+        <v>64</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="H7" s="21">
+        <v>66.5</v>
+      </c>
+      <c r="I7" s="19">
+        <v>1.4500999999999999</v>
+      </c>
+      <c r="J7" s="20">
+        <v>1.1358999999999999</v>
+      </c>
+      <c r="K7" s="21">
+        <v>0.94550000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="6">
+        <v>15</v>
+      </c>
+      <c r="C8" s="6">
+        <v>50</v>
+      </c>
+      <c r="D8" s="6">
+        <v>32</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="H8" s="21">
+        <v>18.75</v>
+      </c>
+      <c r="I8" s="31">
+        <v>1.0931</v>
+      </c>
+      <c r="J8" s="32">
+        <v>0.82979999999999998</v>
+      </c>
+      <c r="K8" s="33">
+        <v>0.96909999999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="29">
+        <v>15</v>
+      </c>
+      <c r="C9" s="29">
+        <v>50</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="29">
+        <v>0.1</v>
+      </c>
+      <c r="G9" s="29">
+        <v>1E-3</v>
+      </c>
+      <c r="H9" s="30">
+        <v>30.88</v>
+      </c>
+      <c r="I9" s="22">
+        <v>1.1484000000000001</v>
+      </c>
+      <c r="J9" s="23">
+        <v>0.88070000000000004</v>
+      </c>
+      <c r="K9" s="24">
+        <v>0.96579999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L14" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>